<commit_message>
KMIP mapping: put hydrogen Other into Domestic|Electricity, not into the totals
Secondary Energy|Hydrogen|Other (nuclear, solar, wind electrolysis in GCAM)
was added to Secondary Energy|Hydrogen and |Domestic, which already contain
it, so the domestic total was too high (kaist9 low_nz 2050: 3348 instead of
2295 ktoe; KMIP25 S1: 11935 instead of 8769). The 2025 submission reports
Other inside Domestic|Electricity; the mapping now does the same.
</commit_message>
<xml_diff>
--- a/kaist/kmip/template/kmip_gcam_mapping_template.xlsx
+++ b/kaist/kmip/template/kmip_gcam_mapping_template.xlsx
@@ -3108,7 +3108,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Secondary Energy|Hydrogen|Other; Secondary Energy|Hydrogen|Import</t>
+          <t>Secondary Energy|Hydrogen|Import</t>
         </is>
       </c>
     </row>
@@ -3131,11 +3131,6 @@
           <t>Secondary Energy|Hydrogen</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Secondary Energy|Hydrogen|Other</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3264,6 +3259,11 @@
       <c r="D152" t="inlineStr">
         <is>
           <t>Secondary Energy|Hydrogen|Electricity</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Secondary Energy|Hydrogen|Other</t>
         </is>
       </c>
     </row>

</xml_diff>